<commit_message>
Update Daily Log Dataset
</commit_message>
<xml_diff>
--- a/12629354.xlsx
+++ b/12629354.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jasmeet kaur\Desktop\Python-MCA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD4A41CF-D1A7-4529-8069-B2B6B5DA8DFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{121FF408-A1D6-4C21-93BF-D229B85FF11B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="77">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -248,6 +248,24 @@
   </si>
   <si>
     <t>Simple and Manageable day.</t>
+  </si>
+  <si>
+    <t>fine</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>A pretty good day.</t>
+  </si>
+  <si>
+    <t>Little bit hectic,but it was good</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> A nice peaceful day off.</t>
+  </si>
+  <si>
+    <t>Simple and Relaxing day.</t>
   </si>
 </sst>
 </file>
@@ -1260,7 +1278,9 @@
       <c r="A11" s="13">
         <v>46252</v>
       </c>
-      <c r="B11" s="14"/>
+      <c r="B11" s="14">
+        <v>420</v>
+      </c>
       <c r="C11" s="14">
         <v>30</v>
       </c>
@@ -1298,93 +1318,187 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+    <row r="12" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="13">
+        <v>46253</v>
+      </c>
+      <c r="B12" s="14">
+        <v>420</v>
+      </c>
+      <c r="C12" s="14">
+        <v>20</v>
+      </c>
+      <c r="D12" s="14">
+        <v>20</v>
+      </c>
+      <c r="E12" s="14">
+        <v>10</v>
+      </c>
+      <c r="F12" s="14">
+        <v>480</v>
+      </c>
+      <c r="G12" s="14">
+        <v>8</v>
+      </c>
+      <c r="H12" s="14">
+        <v>90</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
+        <v>400</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+      <c r="A13" s="13">
+        <v>46254</v>
+      </c>
+      <c r="B13" s="14">
+        <v>420</v>
+      </c>
+      <c r="C13" s="14">
+        <v>30</v>
+      </c>
+      <c r="D13" s="14">
+        <v>60</v>
+      </c>
+      <c r="E13" s="14">
+        <v>10</v>
+      </c>
+      <c r="F13" s="14">
+        <v>180</v>
+      </c>
+      <c r="G13" s="14">
+        <v>3</v>
+      </c>
+      <c r="H13" s="14">
+        <v>120</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>820</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17"/>
+        <v>620</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+      <c r="A14" s="13">
+        <v>46255</v>
+      </c>
+      <c r="B14" s="14">
+        <v>360</v>
+      </c>
+      <c r="C14" s="14">
+        <v>20</v>
+      </c>
+      <c r="D14" s="14">
+        <v>30</v>
+      </c>
+      <c r="E14" s="14">
+        <v>20</v>
+      </c>
+      <c r="F14" s="14">
+        <v>0</v>
+      </c>
+      <c r="G14" s="14">
+        <v>0</v>
+      </c>
+      <c r="H14" s="14">
+        <v>180</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>610</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="17"/>
+        <v>830</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="13"/>
+      <c r="A15" s="13">
+        <v>46256</v>
+      </c>
       <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+      <c r="C15" s="14">
+        <v>10</v>
+      </c>
+      <c r="D15" s="14">
+        <v>30</v>
+      </c>
+      <c r="E15" s="14">
+        <v>60</v>
+      </c>
+      <c r="F15" s="14">
+        <v>0</v>
+      </c>
+      <c r="G15" s="14">
+        <v>0</v>
+      </c>
+      <c r="H15" s="14">
+        <v>180</v>
+      </c>
+      <c r="I15" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>280</v>
+      </c>
+      <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="17"/>
+        <v>1160</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="N15" s="17" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>

</xml_diff>